<commit_message>
XLS and PDF added - Presentation List for Student
</commit_message>
<xml_diff>
--- a/StudentFinalPresentation/XLSFormat/A7125_PresentationList.xlsx
+++ b/StudentFinalPresentation/XLSFormat/A7125_PresentationList.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NeedDO\AZDNU\Projects\AI_Course\ai-management-course\StudentFinalPresentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NeedDO\AZDNU\Projects\AI_Course\ai-management-course\StudentFinalPresentation\XLSFormat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0453BA8-934A-41A6-A70F-7EB5507FBF12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE4CD1D-48D6-4D50-A558-1E20FF59E16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{413F673F-1ABC-494B-BF08-799A1B77560E}"/>
   </bookViews>
@@ -809,6 +809,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -817,12 +823,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1201,6 +1201,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8622F708-9397-4207-8E36-FE0349BECA90}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1212,11 +1215,11 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1243,7 +1246,7 @@
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1266,7 +1269,7 @@
       <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -1289,7 +1292,7 @@
       <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -1312,7 +1315,7 @@
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="3" t="s">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -1335,7 +1338,7 @@
       <c r="E6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="3" t="s">
         <v>69</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -1358,7 +1361,7 @@
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="3" t="s">
         <v>70</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -1381,7 +1384,7 @@
       <c r="E8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="4" t="s">
         <v>71</v>
       </c>
       <c r="G8" s="2" t="s">
@@ -1404,7 +1407,7 @@
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="4" t="s">
         <v>72</v>
       </c>
       <c r="G9" s="2" t="s">
@@ -1427,7 +1430,7 @@
       <c r="E10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="4" t="s">
         <v>74</v>
       </c>
       <c r="G10" s="2" t="s">
@@ -1450,7 +1453,7 @@
       <c r="E11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="3" t="s">
         <v>75</v>
       </c>
       <c r="G11" s="2" t="s">
@@ -1473,7 +1476,7 @@
       <c r="E12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="4" t="s">
         <v>74</v>
       </c>
       <c r="G12" s="2" t="s">
@@ -1496,7 +1499,7 @@
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="3" t="s">
         <v>73</v>
       </c>
       <c r="G13" s="2" t="s">
@@ -1519,7 +1522,7 @@
       <c r="E14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="4" t="s">
         <v>71</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -1542,7 +1545,7 @@
       <c r="E15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G15" s="2" t="s">
@@ -1565,7 +1568,7 @@
       <c r="E16" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="4" t="s">
         <v>72</v>
       </c>
       <c r="G16" s="2" t="s">
@@ -1588,7 +1591,7 @@
       <c r="E17" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="3" t="s">
         <v>75</v>
       </c>
       <c r="G17" s="2" t="s">
@@ -1611,7 +1614,7 @@
       <c r="E18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="3" t="s">
         <v>70</v>
       </c>
       <c r="G18" s="2" t="s">
@@ -1634,7 +1637,7 @@
       <c r="E19" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="3" t="s">
         <v>73</v>
       </c>
       <c r="G19" s="2" t="s">
@@ -1645,6 +1648,7 @@
   <mergeCells count="1">
     <mergeCell ref="B1:D1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>